<commit_message>
Imported pandas library and sorted sheet using that. Bug fixed.
</commit_message>
<xml_diff>
--- a/Excel_MOD/_main.xlsx
+++ b/Excel_MOD/_main.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt formatCode="#.000" numFmtId="164"/>
     <numFmt formatCode="#.00000" numFmtId="165"/>
     <numFmt formatCode="#.0000" numFmtId="166"/>
@@ -29,8 +29,9 @@
     <numFmt formatCode="yyyy/mm/dd" numFmtId="168"/>
     <numFmt formatCode="#.00%" numFmtId="169"/>
     <numFmt formatCode="yyyy-mm-dd h:mm:ss" numFmtId="170"/>
+    <numFmt formatCode="YYYY-MM-DD HH:MM:SS" numFmtId="171"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +57,9 @@
       <family val="2"/>
       <color rgb="FFFF0000"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -91,7 +95,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -99,11 +103,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf applyAlignment="1" borderId="0" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
@@ -235,6 +245,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="170" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="1" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="171" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle builtinId="0" name="Normal" xfId="0"/>
@@ -7132,7 +7146,6 @@
           <t>102 MUIRFIELD WAY</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>CARROLLTON</t>
@@ -7428,7 +7441,6 @@
           <t>12151 FOXTAIL LANE S</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>ROGERS</t>
@@ -7724,7 +7736,6 @@
           <t>48775 KENT COURT</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>NOVI</t>
@@ -8320,7 +8331,6 @@
           <t>6973 TOWNSHIP ROAD 177</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>ZANESFIELD</t>
@@ -8766,7 +8776,6 @@
           <t>8068 NAVARRE PKWY</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
           <t>NAVARRE</t>
@@ -8912,7 +8921,6 @@
           <t>1902 SW 7TH ST</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
           <t>ATKINS</t>
@@ -9358,7 +9366,6 @@
           <t>11 CLUB RIDGE COURT</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
           <t>ELGIN</t>
@@ -9504,7 +9511,6 @@
           <t>202 51ST ST</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
           <t>GRAND JUNCTION</t>
@@ -9950,7 +9956,6 @@
           <t>3607 PARK CT</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr">
         <is>
           <t>GRAPEVINE</t>
@@ -10976,216 +10981,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP2"/>
+  <dimension ref="A1:AP6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>WCOPNB</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="45" t="inlineStr">
         <is>
           <t>ORDNO</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="45" t="inlineStr">
         <is>
           <t>CUSNO</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="45" t="inlineStr">
         <is>
           <t>CUSPO</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="45" t="inlineStr">
         <is>
           <t>PRDNO</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="45" t="inlineStr">
         <is>
           <t>Open Qty</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="45" t="inlineStr">
         <is>
           <t>UNWGT</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="45" t="inlineStr">
         <is>
           <t>Master PK Qty</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="45" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="45" t="inlineStr">
         <is>
           <t>OSNAM</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="45" t="inlineStr">
         <is>
           <t>OSAD1</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="45" t="inlineStr">
         <is>
           <t>OSAD2</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="45" t="inlineStr">
         <is>
           <t>OSADX</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="45" t="inlineStr">
         <is>
           <t>OSAD3</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="45" t="inlineStr">
         <is>
           <t>OSSTA</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="45" t="inlineStr">
         <is>
           <t>EIGWT</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="45" t="inlineStr">
         <is>
           <t>EINWT</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="45" t="inlineStr">
         <is>
           <t>EILNG</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="45" t="inlineStr">
         <is>
           <t>EIWID</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="45" t="inlineStr">
         <is>
           <t>EIHGT</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="45" t="inlineStr">
         <is>
           <t>EIVOL</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="45" t="inlineStr">
         <is>
           <t>EICIN</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="45" t="inlineStr">
         <is>
           <t>OSZIP</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="45" t="inlineStr">
         <is>
           <t>ship via</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="45" t="inlineStr">
         <is>
           <t>freight terms</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="45" t="inlineStr">
         <is>
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="45" t="inlineStr">
         <is>
           <t>PSPDAT</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="45" t="inlineStr">
         <is>
           <t>PSPTIM</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="45" t="inlineStr">
         <is>
           <t>Batch #</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="45" t="inlineStr">
         <is>
           <t>Batch Create Date</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="45" t="inlineStr">
         <is>
           <t>WLINE</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="45" t="inlineStr">
         <is>
           <t>WEFLAG</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="45" t="inlineStr">
         <is>
           <t>WEMAIL</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="45" t="inlineStr">
         <is>
           <t>Ship Via From Special Instructions</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="45" t="inlineStr">
         <is>
           <t>Sched Date</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="45" t="inlineStr">
         <is>
           <t>Account Number</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="45" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="45" t="inlineStr">
         <is>
           <t>SCAC</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="45" t="inlineStr">
         <is>
           <t>GLCODE</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="45" t="inlineStr">
         <is>
           <t>53 FTL QTY</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="45" t="inlineStr">
         <is>
           <t>% Of Trailer</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="45" t="inlineStr">
         <is>
           <t>Customer Name</t>
         </is>
@@ -11194,19 +11199,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>I982673000001UP</t>
+          <t>I977909000001UP</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>982673</v>
+        <v>977909</v>
       </c>
       <c r="C2" t="n">
         <v>67255</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1783041094</t>
-        </is>
+      <c r="D2" t="n">
+        <v>1782693808</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -11229,27 +11232,26 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>JONES          KRISTIN R</t>
+          <t>PROTHRO        TOMICA D</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>7719 MARRISEY LOOP</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>6142577268</t>
-        </is>
+          <t>530 BENTONVILLE LN</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>7709201577</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>GALENA</t>
+          <t>DOUGLASVILLE</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="P2" t="n">
@@ -11273,10 +11275,8 @@
       <c r="V2" t="n">
         <v>5096</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>430217005</t>
-        </is>
+      <c r="W2" t="n">
+        <v>301346304</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -11293,7 +11293,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA2" s="44" t="n">
+      <c r="AA2" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB2" t="n">
@@ -11302,6 +11302,7 @@
       <c r="AC2" t="n">
         <v>0</v>
       </c>
+      <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="n">
         <v>3</v>
       </c>
@@ -11310,13 +11311,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr">
         <is>
           <t>SHIP VIA Ground</t>
         </is>
       </c>
-      <c r="AI2" s="44" t="n">
-        <v>44515</v>
+      <c r="AI2" s="46" t="n">
+        <v>44513</v>
       </c>
       <c r="AJ2" t="n">
         <v>0</v>
@@ -11324,6 +11326,7 @@
       <c r="AK2" t="n">
         <v>0</v>
       </c>
+      <c r="AL2" t="inlineStr"/>
       <c r="AM2" t="inlineStr">
         <is>
           <t>11-70-6755000</t>
@@ -11336,6 +11339,602 @@
         <v>0.0032</v>
       </c>
       <c r="AP2" t="inlineStr">
+        <is>
+          <t>HSN DROPSHIP EDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>I982673000001UP</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>982673</v>
+      </c>
+      <c r="C3" t="n">
+        <v>67255</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1783041094</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PFBE39520</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>146</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>J1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>JONES          KRISTIN R</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>7719 MARRISEY LOOP</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>6142577268</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>GALENA</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>146</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>146</v>
+      </c>
+      <c r="R3" t="n">
+        <v>91</v>
+      </c>
+      <c r="S3" t="n">
+        <v>14</v>
+      </c>
+      <c r="T3" t="n">
+        <v>4</v>
+      </c>
+      <c r="U3" t="n">
+        <v>2.949074</v>
+      </c>
+      <c r="V3" t="n">
+        <v>5096</v>
+      </c>
+      <c r="W3" t="n">
+        <v>430217005</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>PROFILE</t>
+        </is>
+      </c>
+      <c r="AA3" s="46" t="n">
+        <v>44517</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>101853</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>SHIP VIA Ground</t>
+        </is>
+      </c>
+      <c r="AI3" s="46" t="n">
+        <v>44515</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>11-70-6755000</t>
+        </is>
+      </c>
+      <c r="AN3" t="n">
+        <v>310</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>HSN DROPSHIP EDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>I991415000001UP</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>991415</v>
+      </c>
+      <c r="C4" t="n">
+        <v>67255</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1783986879</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PFBE00120</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>58</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>J1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>MCRAE          SHANINA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>5048 BENNING RD SE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>2024124540</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>WASHINGTON</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>58.42</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>58.42</v>
+      </c>
+      <c r="R4" t="n">
+        <v>45.28</v>
+      </c>
+      <c r="S4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="T4" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="U4" t="n">
+        <v>3.243101</v>
+      </c>
+      <c r="V4" t="n">
+        <v>5604.0792</v>
+      </c>
+      <c r="W4" t="n">
+        <v>200195838</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>PROFILE</t>
+        </is>
+      </c>
+      <c r="AA4" s="46" t="n">
+        <v>44517</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>101853</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>SHIP VIA Ground</t>
+        </is>
+      </c>
+      <c r="AI4" s="46" t="n">
+        <v>44519</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>11-70-6755000</t>
+        </is>
+      </c>
+      <c r="AN4" t="n">
+        <v>700</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>HSN DROPSHIP EDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>I991416000001UP</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>991416</v>
+      </c>
+      <c r="C5" t="n">
+        <v>67255</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1784015393</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PFBE09620</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>37</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>DANOWSKY       ANN</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1419 PRESTON CT</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>3182864556</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>BOSSIER CITY</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>37</v>
+      </c>
+      <c r="R5" t="n">
+        <v>45</v>
+      </c>
+      <c r="S5" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="T5" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="U5" t="n">
+        <v>17.213932</v>
+      </c>
+      <c r="V5" t="n">
+        <v>29745.675</v>
+      </c>
+      <c r="W5" t="n">
+        <v>711112267</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>PROFILE</t>
+        </is>
+      </c>
+      <c r="AA5" s="46" t="n">
+        <v>44517</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>101853</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>SHIP VIA Ground</t>
+        </is>
+      </c>
+      <c r="AI5" s="46" t="n">
+        <v>44519</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>11-70-6755000</t>
+        </is>
+      </c>
+      <c r="AN5" t="n">
+        <v>720</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>HSN DROPSHIP EDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>I991418000001UP</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>991418</v>
+      </c>
+      <c r="C6" t="n">
+        <v>67255</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1784074866</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PFBE19720</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>68</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>GRAY           SUZANNE</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2510 US HIGHWAY 199</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SPC 7C</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>9162005971</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>CRESCENT CITY</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>68.34</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>68.34</v>
+      </c>
+      <c r="R6" t="n">
+        <v>46.46</v>
+      </c>
+      <c r="S6" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="T6" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="U6" t="n">
+        <v>4.314074</v>
+      </c>
+      <c r="V6" t="n">
+        <v>7454.720716</v>
+      </c>
+      <c r="W6" t="n">
+        <v>955319320</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>PROFILE</t>
+        </is>
+      </c>
+      <c r="AA6" s="46" t="n">
+        <v>44517</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>101853</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>SHIP VIA Ground</t>
+        </is>
+      </c>
+      <c r="AI6" s="46" t="n">
+        <v>44519</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>11-70-6755000</t>
+        </is>
+      </c>
+      <c r="AN6" t="n">
+        <v>480</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="AP6" t="inlineStr">
         <is>
           <t>HSN DROPSHIP EDI</t>
         </is>
@@ -11613,7 +12212,6 @@
           <t>223 N WHITMAN AVE</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>ROSALIA</t>
@@ -11759,7 +12357,6 @@
           <t>2402 SYLVAN DR</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>ABILENE</t>
@@ -11905,7 +12502,6 @@
           <t>1015 S 1960 E</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>SPRINGVILLE</t>
@@ -12051,7 +12647,6 @@
           <t>223 N WHITMAN AVE</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>ROSALIA</t>
@@ -12197,7 +12792,6 @@
           <t>2402 SYLVAN DR</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>ABILENE</t>
@@ -12343,7 +12937,6 @@
           <t>8540 DUNDEE TER</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>MIAMI LAKES</t>
@@ -12489,7 +13082,6 @@
           <t>26 ESTELLA DR</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>FLEMINGTON</t>
@@ -12635,7 +13227,6 @@
           <t>1213 AMBER DRIVE</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>LOGANVILLE</t>
@@ -12781,7 +13372,6 @@
           <t>2 BEECHWOOD LN</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>MILLSTONE TWP</t>
@@ -12927,7 +13517,6 @@
           <t>441 11TH ST S</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>WISCONSIN RAPIDS</t>
@@ -13073,7 +13662,6 @@
           <t>27 LAWRENCE ST</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>HAVERHILL</t>
@@ -13219,7 +13807,6 @@
           <t>17507 76TH ST W</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>REYNOLDS</t>
@@ -13365,7 +13952,6 @@
           <t>5230 CRABAPPLE CT</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>LOVELAND</t>
@@ -13516,7 +14102,6 @@
           <t>APT L201</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>BOISE</t>
@@ -13662,7 +14247,6 @@
           <t>10786 HILLSBORO CIR</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>PARKER</t>
@@ -14034,7 +14618,6 @@
           <t>277 WETUMKA LN</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>EL PASO</t>
@@ -14180,7 +14763,6 @@
           <t>716 SARAJANE LN</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>LAS VEGAS</t>
@@ -14326,7 +14908,6 @@
           <t>277 WETUMKA LN</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>EL PASO</t>
@@ -14472,7 +15053,6 @@
           <t>716 SARAJANE LN</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>LAS VEGAS</t>
@@ -14618,7 +15198,6 @@
           <t>3319 W IAN DR</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>LAVEEN</t>
@@ -14769,7 +15348,6 @@
           <t>13527 SUNBURST ST</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>ARLETA</t>

</xml_diff>

<commit_message>
Added split order fill function. (Need?) to do blue for kits next.
</commit_message>
<xml_diff>
--- a/Excel_MOD/_main.xlsx
+++ b/Excel_MOD/_main.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="18000" windowWidth="28800" xWindow="0" yWindow="0"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="15330" windowWidth="23250" xWindow="2355" yWindow="45"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId1"/>
@@ -58,7 +58,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -92,8 +92,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF66FF66"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="008497b0"/>
         <bgColor rgb="008497b0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0066FF66"/>
+        <bgColor rgb="0066FF66"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf applyAlignment="1" borderId="0" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
@@ -240,91 +252,21 @@
     <xf applyAlignment="1" borderId="0" fillId="4" fontId="3" numFmtId="169" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf applyAlignment="1" borderId="0" fillId="7" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf applyAlignment="1" borderId="0" fillId="7" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="170" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="7" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="9" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="8" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle builtinId="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF424649"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -596,49 +538,49 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AP2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col bestFit="1" customWidth="1" max="1" min="1" width="16.1640625"/>
-    <col bestFit="1" customWidth="1" max="3" min="2" width="7.83203125"/>
-    <col bestFit="1" customWidth="1" max="4" min="4" width="16.1640625"/>
-    <col bestFit="1" customWidth="1" max="5" min="5" width="14.5"/>
-    <col bestFit="1" customWidth="1" max="6" min="6" width="9.6640625"/>
-    <col bestFit="1" customWidth="1" max="7" min="7" width="8.5"/>
-    <col bestFit="1" customWidth="1" max="8" min="8" width="13.5"/>
-    <col bestFit="1" customWidth="1" max="9" min="9" width="9.1640625"/>
-    <col bestFit="1" customWidth="1" max="11" min="10" width="26.83203125"/>
+    <col bestFit="1" customWidth="1" max="1" min="1" width="16.140625"/>
+    <col bestFit="1" customWidth="1" max="3" min="2" width="7.85546875"/>
+    <col bestFit="1" customWidth="1" max="4" min="4" width="16.140625"/>
+    <col bestFit="1" customWidth="1" max="5" min="5" width="14.42578125"/>
+    <col bestFit="1" customWidth="1" max="6" min="6" width="9.7109375"/>
+    <col bestFit="1" customWidth="1" max="7" min="7" width="8.42578125"/>
+    <col bestFit="1" customWidth="1" max="8" min="8" width="13.42578125"/>
+    <col bestFit="1" customWidth="1" max="9" min="9" width="9.140625"/>
+    <col bestFit="1" customWidth="1" max="11" min="10" width="26.85546875"/>
     <col bestFit="1" customWidth="1" max="12" min="12" width="27"/>
-    <col bestFit="1" customWidth="1" max="13" min="13" width="30.83203125"/>
-    <col bestFit="1" customWidth="1" max="14" min="14" width="20.1640625"/>
-    <col bestFit="1" customWidth="1" max="15" min="15" width="7.33203125"/>
-    <col bestFit="1" customWidth="1" max="17" min="16" width="10.5"/>
-    <col bestFit="1" customWidth="1" max="18" min="18" width="9.5"/>
-    <col bestFit="1" customWidth="1" max="20" min="19" width="8.5"/>
-    <col bestFit="1" customWidth="1" max="21" min="21" width="10.5"/>
-    <col bestFit="1" customWidth="1" max="22" min="22" width="13.33203125"/>
-    <col bestFit="1" customWidth="1" max="23" min="23" width="11.33203125"/>
-    <col bestFit="1" customWidth="1" max="24" min="24" width="9.6640625"/>
-    <col bestFit="1" customWidth="1" max="25" min="25" width="12.83203125"/>
-    <col bestFit="1" customWidth="1" max="26" min="26" width="8.6640625"/>
-    <col bestFit="1" customWidth="1" max="27" min="27" width="11.6640625"/>
-    <col bestFit="1" customWidth="1" max="28" min="28" width="7.83203125"/>
-    <col bestFit="1" customWidth="1" max="29" min="29" width="10.6640625"/>
-    <col bestFit="1" customWidth="1" max="30" min="30" width="16.83203125"/>
-    <col bestFit="1" customWidth="1" max="31" min="31" width="7.33203125"/>
-    <col bestFit="1" customWidth="1" max="32" min="32" width="8.83203125"/>
-    <col bestFit="1" customWidth="1" max="33" min="33" width="31.1640625"/>
-    <col bestFit="1" customWidth="1" max="34" min="34" width="35.1640625"/>
-    <col bestFit="1" customWidth="1" max="35" min="35" width="11.6640625"/>
-    <col bestFit="1" customWidth="1" max="36" min="36" width="15.5"/>
-    <col bestFit="1" customWidth="1" max="37" min="37" width="5.1640625"/>
-    <col bestFit="1" customWidth="1" max="38" min="38" width="7.1640625"/>
-    <col bestFit="1" customWidth="1" max="39" min="39" width="13.83203125"/>
-    <col bestFit="1" customWidth="1" max="40" min="40" width="11.33203125"/>
-    <col bestFit="1" customWidth="1" max="41" min="41" width="11.6640625"/>
-    <col bestFit="1" customWidth="1" max="42" min="42" width="27.5"/>
+    <col bestFit="1" customWidth="1" max="13" min="13" width="30.85546875"/>
+    <col bestFit="1" customWidth="1" max="14" min="14" width="20.140625"/>
+    <col bestFit="1" customWidth="1" max="15" min="15" width="7.28515625"/>
+    <col bestFit="1" customWidth="1" max="17" min="16" width="10.42578125"/>
+    <col bestFit="1" customWidth="1" max="18" min="18" width="9.42578125"/>
+    <col bestFit="1" customWidth="1" max="20" min="19" width="8.42578125"/>
+    <col bestFit="1" customWidth="1" max="21" min="21" width="10.42578125"/>
+    <col bestFit="1" customWidth="1" max="22" min="22" width="13.28515625"/>
+    <col bestFit="1" customWidth="1" max="23" min="23" width="11.28515625"/>
+    <col bestFit="1" customWidth="1" max="24" min="24" width="9.7109375"/>
+    <col bestFit="1" customWidth="1" max="25" min="25" width="12.85546875"/>
+    <col bestFit="1" customWidth="1" max="26" min="26" width="8.7109375"/>
+    <col bestFit="1" customWidth="1" max="27" min="27" width="11.7109375"/>
+    <col bestFit="1" customWidth="1" max="28" min="28" width="7.85546875"/>
+    <col bestFit="1" customWidth="1" max="29" min="29" width="10.7109375"/>
+    <col bestFit="1" customWidth="1" max="30" min="30" width="16.85546875"/>
+    <col bestFit="1" customWidth="1" max="31" min="31" width="7.28515625"/>
+    <col bestFit="1" customWidth="1" max="32" min="32" width="8.85546875"/>
+    <col bestFit="1" customWidth="1" max="33" min="33" width="31.140625"/>
+    <col bestFit="1" customWidth="1" max="34" min="34" width="35.140625"/>
+    <col bestFit="1" customWidth="1" max="35" min="35" width="11.7109375"/>
+    <col bestFit="1" customWidth="1" max="36" min="36" width="15.42578125"/>
+    <col bestFit="1" customWidth="1" max="37" min="37" width="5.140625"/>
+    <col bestFit="1" customWidth="1" max="38" min="38" width="7.140625"/>
+    <col bestFit="1" customWidth="1" max="39" min="39" width="13.85546875"/>
+    <col bestFit="1" customWidth="1" max="40" min="40" width="11.28515625"/>
+    <col bestFit="1" customWidth="1" max="41" min="41" width="11.7109375"/>
+    <col bestFit="1" customWidth="1" max="42" min="42" width="27.42578125"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row customHeight="1" ht="16.5" r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>WCOPNB</t>
@@ -850,7 +792,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row customHeight="1" ht="16.5" r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>I989790000001RT</t>
@@ -1000,6 +942,493 @@
         </is>
       </c>
     </row>
+    <row customHeight="1" ht="16.5" r="3"/>
+    <row customHeight="1" ht="16.5" r="4"/>
+    <row customHeight="1" ht="16.5" r="5"/>
+    <row customHeight="1" ht="16.5" r="6"/>
+    <row customHeight="1" ht="16.5" r="7"/>
+    <row customHeight="1" ht="16.5" r="8"/>
+    <row customHeight="1" ht="16.5" r="9"/>
+    <row customHeight="1" ht="16.5" r="10"/>
+    <row customHeight="1" ht="16.5" r="11"/>
+    <row customHeight="1" ht="16.5" r="12"/>
+    <row customHeight="1" ht="16.5" r="13"/>
+    <row customHeight="1" ht="16.5" r="14"/>
+    <row customHeight="1" ht="16.5" r="15"/>
+    <row customHeight="1" ht="16.5" r="16"/>
+    <row customHeight="1" ht="16.5" r="17"/>
+    <row customHeight="1" ht="16.5" r="18"/>
+    <row customHeight="1" ht="16.5" r="19"/>
+    <row customHeight="1" ht="16.5" r="20"/>
+    <row customHeight="1" ht="16.5" r="21"/>
+    <row customHeight="1" ht="16.5" r="22"/>
+    <row customHeight="1" ht="16.5" r="23"/>
+    <row customHeight="1" ht="16.5" r="24"/>
+    <row customHeight="1" ht="16.5" r="25"/>
+    <row customHeight="1" ht="16.5" r="26"/>
+    <row customHeight="1" ht="16.5" r="27"/>
+    <row customHeight="1" ht="16.5" r="28"/>
+    <row customHeight="1" ht="16.5" r="29"/>
+    <row customHeight="1" ht="16.5" r="30"/>
+    <row customHeight="1" ht="16.5" r="31"/>
+    <row customHeight="1" ht="16.5" r="32"/>
+    <row customHeight="1" ht="16.5" r="33"/>
+    <row customHeight="1" ht="16.5" r="34"/>
+    <row customHeight="1" ht="16.5" r="35"/>
+    <row customHeight="1" ht="16.5" r="36"/>
+    <row customHeight="1" ht="16.5" r="37"/>
+    <row customHeight="1" ht="16.5" r="38"/>
+    <row customHeight="1" ht="16.5" r="39"/>
+    <row customHeight="1" ht="16.5" r="40"/>
+    <row customHeight="1" ht="16.5" r="41"/>
+    <row customHeight="1" ht="16.5" r="42"/>
+    <row customHeight="1" ht="16.5" r="43"/>
+    <row customHeight="1" ht="16.5" r="44"/>
+    <row customHeight="1" ht="16.5" r="45"/>
+    <row customHeight="1" ht="16.5" r="46"/>
+    <row customHeight="1" ht="16.5" r="47"/>
+    <row customHeight="1" ht="16.5" r="48"/>
+    <row customHeight="1" ht="16.5" r="49"/>
+    <row customHeight="1" ht="16.5" r="50"/>
+    <row customHeight="1" ht="16.5" r="51"/>
+    <row customHeight="1" ht="16.5" r="52"/>
+    <row customHeight="1" ht="16.5" r="53"/>
+    <row customHeight="1" ht="16.5" r="54"/>
+    <row customHeight="1" ht="16.5" r="55"/>
+    <row customHeight="1" ht="16.5" r="56"/>
+    <row customHeight="1" ht="16.5" r="57"/>
+    <row customHeight="1" ht="16.5" r="58"/>
+    <row customHeight="1" ht="16.5" r="59"/>
+    <row customHeight="1" ht="16.5" r="60"/>
+    <row customHeight="1" ht="16.5" r="61"/>
+    <row customHeight="1" ht="16.5" r="62"/>
+    <row customHeight="1" ht="16.5" r="63"/>
+    <row customHeight="1" ht="16.5" r="64"/>
+    <row customHeight="1" ht="16.5" r="65"/>
+    <row customHeight="1" ht="16.5" r="66"/>
+    <row customHeight="1" ht="16.5" r="67"/>
+    <row customHeight="1" ht="16.5" r="68"/>
+    <row customHeight="1" ht="16.5" r="69"/>
+    <row customHeight="1" ht="16.5" r="70"/>
+    <row customHeight="1" ht="16.5" r="71"/>
+    <row customHeight="1" ht="16.5" r="72"/>
+    <row customHeight="1" ht="16.5" r="73"/>
+    <row customHeight="1" ht="16.5" r="74"/>
+    <row customHeight="1" ht="16.5" r="75"/>
+    <row customHeight="1" ht="16.5" r="76"/>
+    <row customHeight="1" ht="16.5" r="77"/>
+    <row customHeight="1" ht="16.5" r="78"/>
+    <row customHeight="1" ht="16.5" r="79"/>
+    <row customHeight="1" ht="16.5" r="80"/>
+    <row customHeight="1" ht="16.5" r="81"/>
+    <row customHeight="1" ht="16.5" r="82"/>
+    <row customHeight="1" ht="16.5" r="83"/>
+    <row customHeight="1" ht="16.5" r="84"/>
+    <row customHeight="1" ht="16.5" r="85"/>
+    <row customHeight="1" ht="16.5" r="86"/>
+    <row customHeight="1" ht="16.5" r="87"/>
+    <row customHeight="1" ht="16.5" r="88"/>
+    <row customHeight="1" ht="16.5" r="89"/>
+    <row customHeight="1" ht="16.5" r="90"/>
+    <row customHeight="1" ht="16.5" r="91"/>
+    <row customHeight="1" ht="16.5" r="92"/>
+    <row customHeight="1" ht="16.5" r="93"/>
+    <row customHeight="1" ht="16.5" r="94"/>
+    <row customHeight="1" ht="16.5" r="95"/>
+    <row customHeight="1" ht="16.5" r="96"/>
+    <row customHeight="1" ht="16.5" r="97"/>
+    <row customHeight="1" ht="16.5" r="98"/>
+    <row customHeight="1" ht="16.5" r="99"/>
+    <row customHeight="1" ht="16.5" r="100"/>
+    <row customHeight="1" ht="16.5" r="101"/>
+    <row customHeight="1" ht="16.5" r="102"/>
+    <row customHeight="1" ht="16.5" r="103"/>
+    <row customHeight="1" ht="16.5" r="104"/>
+    <row customHeight="1" ht="16.5" r="105"/>
+    <row customHeight="1" ht="16.5" r="106"/>
+    <row customHeight="1" ht="16.5" r="107"/>
+    <row customHeight="1" ht="16.5" r="108"/>
+    <row customHeight="1" ht="16.5" r="109"/>
+    <row customHeight="1" ht="16.5" r="110"/>
+    <row customHeight="1" ht="16.5" r="111"/>
+    <row customHeight="1" ht="16.5" r="112"/>
+    <row customHeight="1" ht="16.5" r="113"/>
+    <row customHeight="1" ht="16.5" r="114"/>
+    <row customHeight="1" ht="16.5" r="115"/>
+    <row customHeight="1" ht="16.5" r="116"/>
+    <row customHeight="1" ht="16.5" r="117"/>
+    <row customHeight="1" ht="16.5" r="118"/>
+    <row customHeight="1" ht="16.5" r="119"/>
+    <row customHeight="1" ht="16.5" r="120"/>
+    <row customHeight="1" ht="16.5" r="121"/>
+    <row customHeight="1" ht="16.5" r="122"/>
+    <row customHeight="1" ht="16.5" r="123"/>
+    <row customHeight="1" ht="16.5" r="124"/>
+    <row customHeight="1" ht="16.5" r="125"/>
+    <row customHeight="1" ht="16.5" r="126"/>
+    <row customHeight="1" ht="16.5" r="127"/>
+    <row customHeight="1" ht="16.5" r="128"/>
+    <row customHeight="1" ht="16.5" r="129"/>
+    <row customHeight="1" ht="16.5" r="130"/>
+    <row customHeight="1" ht="16.5" r="131"/>
+    <row customHeight="1" ht="16.5" r="132"/>
+    <row customHeight="1" ht="16.5" r="133"/>
+    <row customHeight="1" ht="16.5" r="134"/>
+    <row customHeight="1" ht="16.5" r="135"/>
+    <row customHeight="1" ht="16.5" r="136"/>
+    <row customHeight="1" ht="16.5" r="137"/>
+    <row customHeight="1" ht="16.5" r="138"/>
+    <row customHeight="1" ht="16.5" r="139"/>
+    <row customHeight="1" ht="16.5" r="140"/>
+    <row customHeight="1" ht="16.5" r="141"/>
+    <row customHeight="1" ht="16.5" r="142"/>
+    <row customHeight="1" ht="16.5" r="143"/>
+    <row customHeight="1" ht="16.5" r="144"/>
+    <row customHeight="1" ht="16.5" r="145"/>
+    <row customHeight="1" ht="16.5" r="146"/>
+    <row customHeight="1" ht="16.5" r="147"/>
+    <row customHeight="1" ht="16.5" r="148"/>
+    <row customHeight="1" ht="16.5" r="149"/>
+    <row customHeight="1" ht="16.5" r="150"/>
+    <row customHeight="1" ht="16.5" r="151"/>
+    <row customHeight="1" ht="16.5" r="152"/>
+    <row customHeight="1" ht="16.5" r="153"/>
+    <row customHeight="1" ht="16.5" r="154"/>
+    <row customHeight="1" ht="16.5" r="155"/>
+    <row customHeight="1" ht="16.5" r="156"/>
+    <row customHeight="1" ht="16.5" r="157"/>
+    <row customHeight="1" ht="16.5" r="158"/>
+    <row customHeight="1" ht="16.5" r="159"/>
+    <row customHeight="1" ht="16.5" r="160"/>
+    <row customHeight="1" ht="16.5" r="161"/>
+    <row customHeight="1" ht="16.5" r="162"/>
+    <row customHeight="1" ht="16.5" r="163"/>
+    <row customHeight="1" ht="16.5" r="164"/>
+    <row customHeight="1" ht="16.5" r="165"/>
+    <row customHeight="1" ht="16.5" r="166"/>
+    <row customHeight="1" ht="16.5" r="167"/>
+    <row customHeight="1" ht="16.5" r="168"/>
+    <row customHeight="1" ht="16.5" r="169"/>
+    <row customHeight="1" ht="16.5" r="170"/>
+    <row customHeight="1" ht="16.5" r="171"/>
+    <row customHeight="1" ht="16.5" r="172"/>
+    <row customHeight="1" ht="16.5" r="173"/>
+    <row customHeight="1" ht="16.5" r="174"/>
+    <row customHeight="1" ht="16.5" r="175"/>
+    <row customHeight="1" ht="16.5" r="176"/>
+    <row customHeight="1" ht="16.5" r="177"/>
+    <row customHeight="1" ht="16.5" r="178"/>
+    <row customHeight="1" ht="16.5" r="179"/>
+    <row customHeight="1" ht="16.5" r="180"/>
+    <row customHeight="1" ht="16.5" r="181"/>
+    <row customHeight="1" ht="16.5" r="182"/>
+    <row customHeight="1" ht="16.5" r="183"/>
+    <row customHeight="1" ht="16.5" r="184"/>
+    <row customHeight="1" ht="16.5" r="185"/>
+    <row customHeight="1" ht="16.5" r="186"/>
+    <row customHeight="1" ht="16.5" r="187"/>
+    <row customHeight="1" ht="16.5" r="188"/>
+    <row customHeight="1" ht="16.5" r="189"/>
+    <row customHeight="1" ht="16.5" r="190"/>
+    <row customHeight="1" ht="16.5" r="191"/>
+    <row customHeight="1" ht="16.5" r="192"/>
+    <row customHeight="1" ht="16.5" r="193"/>
+    <row customHeight="1" ht="16.5" r="194"/>
+    <row customHeight="1" ht="16.5" r="195"/>
+    <row customHeight="1" ht="16.5" r="196"/>
+    <row customHeight="1" ht="16.5" r="197"/>
+    <row customHeight="1" ht="16.5" r="198"/>
+    <row customHeight="1" ht="16.5" r="199"/>
+    <row customHeight="1" ht="16.5" r="200"/>
+    <row customHeight="1" ht="16.5" r="201"/>
+    <row customHeight="1" ht="16.5" r="202"/>
+    <row customHeight="1" ht="16.5" r="203"/>
+    <row customHeight="1" ht="16.5" r="204"/>
+    <row customHeight="1" ht="16.5" r="205"/>
+    <row customHeight="1" ht="16.5" r="206"/>
+    <row customHeight="1" ht="16.5" r="207"/>
+    <row customHeight="1" ht="16.5" r="208"/>
+    <row customHeight="1" ht="16.5" r="209"/>
+    <row customHeight="1" ht="16.5" r="210"/>
+    <row customHeight="1" ht="16.5" r="211"/>
+    <row customHeight="1" ht="16.5" r="212"/>
+    <row customHeight="1" ht="16.5" r="213"/>
+    <row customHeight="1" ht="16.5" r="214"/>
+    <row customHeight="1" ht="16.5" r="215"/>
+    <row customHeight="1" ht="16.5" r="216"/>
+    <row customHeight="1" ht="16.5" r="217"/>
+    <row customHeight="1" ht="16.5" r="218"/>
+    <row customHeight="1" ht="16.5" r="219"/>
+    <row customHeight="1" ht="16.5" r="220"/>
+    <row customHeight="1" ht="16.5" r="221"/>
+    <row customHeight="1" ht="16.5" r="222"/>
+    <row customHeight="1" ht="16.5" r="223"/>
+    <row customHeight="1" ht="16.5" r="224"/>
+    <row customHeight="1" ht="16.5" r="225"/>
+    <row customHeight="1" ht="16.5" r="226"/>
+    <row customHeight="1" ht="16.5" r="227"/>
+    <row customHeight="1" ht="16.5" r="228"/>
+    <row customHeight="1" ht="16.5" r="229"/>
+    <row customHeight="1" ht="16.5" r="230"/>
+    <row customHeight="1" ht="16.5" r="231"/>
+    <row customHeight="1" ht="16.5" r="232"/>
+    <row customHeight="1" ht="16.5" r="233"/>
+    <row customHeight="1" ht="16.5" r="234"/>
+    <row customHeight="1" ht="16.5" r="235"/>
+    <row customHeight="1" ht="16.5" r="236"/>
+    <row customHeight="1" ht="16.5" r="237"/>
+    <row customHeight="1" ht="16.5" r="238"/>
+    <row customHeight="1" ht="16.5" r="239"/>
+    <row customHeight="1" ht="16.5" r="240"/>
+    <row customHeight="1" ht="16.5" r="241"/>
+    <row customHeight="1" ht="16.5" r="242"/>
+    <row customHeight="1" ht="16.5" r="243"/>
+    <row customHeight="1" ht="16.5" r="244"/>
+    <row customHeight="1" ht="16.5" r="245"/>
+    <row customHeight="1" ht="16.5" r="246"/>
+    <row customHeight="1" ht="16.5" r="247"/>
+    <row customHeight="1" ht="16.5" r="248"/>
+    <row customHeight="1" ht="16.5" r="249"/>
+    <row customHeight="1" ht="16.5" r="250"/>
+    <row customHeight="1" ht="16.5" r="251"/>
+    <row customHeight="1" ht="16.5" r="252"/>
+    <row customHeight="1" ht="16.5" r="253"/>
+    <row customHeight="1" ht="16.5" r="254"/>
+    <row customHeight="1" ht="16.5" r="255"/>
+    <row customHeight="1" ht="16.5" r="256"/>
+    <row customHeight="1" ht="16.5" r="257"/>
+    <row customHeight="1" ht="16.5" r="258"/>
+    <row customHeight="1" ht="16.5" r="259"/>
+    <row customHeight="1" ht="16.5" r="260"/>
+    <row customHeight="1" ht="16.5" r="261"/>
+    <row customHeight="1" ht="16.5" r="262"/>
+    <row customHeight="1" ht="16.5" r="263"/>
+    <row customHeight="1" ht="16.5" r="264"/>
+    <row customHeight="1" ht="16.5" r="265"/>
+    <row customHeight="1" ht="16.5" r="266"/>
+    <row customHeight="1" ht="16.5" r="267"/>
+    <row customHeight="1" ht="16.5" r="268"/>
+    <row customHeight="1" ht="16.5" r="269"/>
+    <row customHeight="1" ht="16.5" r="270"/>
+    <row customHeight="1" ht="16.5" r="271"/>
+    <row customHeight="1" ht="16.5" r="272"/>
+    <row customHeight="1" ht="16.5" r="273"/>
+    <row customHeight="1" ht="16.5" r="274"/>
+    <row customHeight="1" ht="16.5" r="275"/>
+    <row customHeight="1" ht="16.5" r="276"/>
+    <row customHeight="1" ht="16.5" r="277"/>
+    <row customHeight="1" ht="16.5" r="278"/>
+    <row customHeight="1" ht="16.5" r="279"/>
+    <row customHeight="1" ht="16.5" r="280"/>
+    <row customHeight="1" ht="16.5" r="281"/>
+    <row customHeight="1" ht="16.5" r="282"/>
+    <row customHeight="1" ht="16.5" r="283"/>
+    <row customHeight="1" ht="16.5" r="284"/>
+    <row customHeight="1" ht="16.5" r="285"/>
+    <row customHeight="1" ht="16.5" r="286"/>
+    <row customHeight="1" ht="16.5" r="287"/>
+    <row customHeight="1" ht="16.5" r="288"/>
+    <row customHeight="1" ht="16.5" r="289"/>
+    <row customHeight="1" ht="16.5" r="290"/>
+    <row customHeight="1" ht="16.5" r="291"/>
+    <row customHeight="1" ht="16.5" r="292"/>
+    <row customHeight="1" ht="16.5" r="293"/>
+    <row customHeight="1" ht="16.5" r="294"/>
+    <row customHeight="1" ht="16.5" r="295"/>
+    <row customHeight="1" ht="16.5" r="296"/>
+    <row customHeight="1" ht="16.5" r="297"/>
+    <row customHeight="1" ht="16.5" r="298"/>
+    <row customHeight="1" ht="16.5" r="299"/>
+    <row customHeight="1" ht="16.5" r="300"/>
+    <row customHeight="1" ht="16.5" r="301"/>
+    <row customHeight="1" ht="16.5" r="302"/>
+    <row customHeight="1" ht="16.5" r="303"/>
+    <row customHeight="1" ht="16.5" r="304"/>
+    <row customHeight="1" ht="16.5" r="305"/>
+    <row customHeight="1" ht="16.5" r="306"/>
+    <row customHeight="1" ht="16.5" r="307"/>
+    <row customHeight="1" ht="16.5" r="308"/>
+    <row customHeight="1" ht="16.5" r="309"/>
+    <row customHeight="1" ht="16.5" r="310"/>
+    <row customHeight="1" ht="16.5" r="311"/>
+    <row customHeight="1" ht="16.5" r="312"/>
+    <row customHeight="1" ht="16.5" r="313"/>
+    <row customHeight="1" ht="16.5" r="314"/>
+    <row customHeight="1" ht="16.5" r="315"/>
+    <row customHeight="1" ht="16.5" r="316"/>
+    <row customHeight="1" ht="16.5" r="317"/>
+    <row customHeight="1" ht="16.5" r="318"/>
+    <row customHeight="1" ht="16.5" r="319"/>
+    <row customHeight="1" ht="16.5" r="320"/>
+    <row customHeight="1" ht="16.5" r="321"/>
+    <row customHeight="1" ht="16.5" r="322"/>
+    <row customHeight="1" ht="16.5" r="323"/>
+    <row customHeight="1" ht="16.5" r="324"/>
+    <row customHeight="1" ht="16.5" r="325"/>
+    <row customHeight="1" ht="16.5" r="326"/>
+    <row customHeight="1" ht="16.5" r="327"/>
+    <row customHeight="1" ht="16.5" r="328"/>
+    <row customHeight="1" ht="16.5" r="329"/>
+    <row customHeight="1" ht="16.5" r="330"/>
+    <row customHeight="1" ht="16.5" r="331"/>
+    <row customHeight="1" ht="16.5" r="332"/>
+    <row customHeight="1" ht="16.5" r="333"/>
+    <row customHeight="1" ht="16.5" r="334"/>
+    <row customHeight="1" ht="16.5" r="335"/>
+    <row customHeight="1" ht="16.5" r="336"/>
+    <row customHeight="1" ht="16.5" r="337"/>
+    <row customHeight="1" ht="16.5" r="338"/>
+    <row customHeight="1" ht="16.5" r="339"/>
+    <row customHeight="1" ht="16.5" r="340"/>
+    <row customHeight="1" ht="16.5" r="341"/>
+    <row customHeight="1" ht="16.5" r="342"/>
+    <row customHeight="1" ht="16.5" r="343"/>
+    <row customHeight="1" ht="16.5" r="344"/>
+    <row customHeight="1" ht="16.5" r="345"/>
+    <row customHeight="1" ht="16.5" r="346"/>
+    <row customHeight="1" ht="16.5" r="347"/>
+    <row customHeight="1" ht="16.5" r="348"/>
+    <row customHeight="1" ht="16.5" r="349"/>
+    <row customHeight="1" ht="16.5" r="350"/>
+    <row customHeight="1" ht="16.5" r="351"/>
+    <row customHeight="1" ht="16.5" r="352"/>
+    <row customHeight="1" ht="16.5" r="353"/>
+    <row customHeight="1" ht="16.5" r="354"/>
+    <row customHeight="1" ht="16.5" r="355"/>
+    <row customHeight="1" ht="16.5" r="356"/>
+    <row customHeight="1" ht="16.5" r="357"/>
+    <row customHeight="1" ht="16.5" r="358"/>
+    <row customHeight="1" ht="16.5" r="359"/>
+    <row customHeight="1" ht="16.5" r="360"/>
+    <row customHeight="1" ht="16.5" r="361"/>
+    <row customHeight="1" ht="16.5" r="362"/>
+    <row customHeight="1" ht="16.5" r="363"/>
+    <row customHeight="1" ht="16.5" r="364"/>
+    <row customHeight="1" ht="16.5" r="365"/>
+    <row customHeight="1" ht="16.5" r="366"/>
+    <row customHeight="1" ht="16.5" r="367"/>
+    <row customHeight="1" ht="16.5" r="368"/>
+    <row customHeight="1" ht="16.5" r="369"/>
+    <row customHeight="1" ht="16.5" r="370"/>
+    <row customHeight="1" ht="16.5" r="371"/>
+    <row customHeight="1" ht="16.5" r="372"/>
+    <row customHeight="1" ht="16.5" r="373"/>
+    <row customHeight="1" ht="16.5" r="374"/>
+    <row customHeight="1" ht="16.5" r="375"/>
+    <row customHeight="1" ht="16.5" r="376"/>
+    <row customHeight="1" ht="16.5" r="377"/>
+    <row customHeight="1" ht="16.5" r="378"/>
+    <row customHeight="1" ht="16.5" r="379"/>
+    <row customHeight="1" ht="16.5" r="380"/>
+    <row customHeight="1" ht="16.5" r="381"/>
+    <row customHeight="1" ht="16.5" r="382"/>
+    <row customHeight="1" ht="16.5" r="383"/>
+    <row customHeight="1" ht="16.5" r="384"/>
+    <row customHeight="1" ht="16.5" r="385"/>
+    <row customHeight="1" ht="16.5" r="386"/>
+    <row customHeight="1" ht="16.5" r="387"/>
+    <row customHeight="1" ht="16.5" r="388"/>
+    <row customHeight="1" ht="16.5" r="389"/>
+    <row customHeight="1" ht="16.5" r="390"/>
+    <row customHeight="1" ht="16.5" r="391"/>
+    <row customHeight="1" ht="16.5" r="392"/>
+    <row customHeight="1" ht="16.5" r="393"/>
+    <row customHeight="1" ht="16.5" r="394"/>
+    <row customHeight="1" ht="16.5" r="395"/>
+    <row customHeight="1" ht="16.5" r="396"/>
+    <row customHeight="1" ht="16.5" r="397"/>
+    <row customHeight="1" ht="16.5" r="398"/>
+    <row customHeight="1" ht="16.5" r="399"/>
+    <row customHeight="1" ht="16.5" r="400"/>
+    <row customHeight="1" ht="16.5" r="401"/>
+    <row customHeight="1" ht="16.5" r="402"/>
+    <row customHeight="1" ht="16.5" r="403"/>
+    <row customHeight="1" ht="16.5" r="404"/>
+    <row customHeight="1" ht="16.5" r="405"/>
+    <row customHeight="1" ht="16.5" r="406"/>
+    <row customHeight="1" ht="16.5" r="407"/>
+    <row customHeight="1" ht="16.5" r="408"/>
+    <row customHeight="1" ht="16.5" r="409"/>
+    <row customHeight="1" ht="16.5" r="410"/>
+    <row customHeight="1" ht="16.5" r="411"/>
+    <row customHeight="1" ht="16.5" r="412"/>
+    <row customHeight="1" ht="16.5" r="413"/>
+    <row customHeight="1" ht="16.5" r="414"/>
+    <row customHeight="1" ht="16.5" r="415"/>
+    <row customHeight="1" ht="16.5" r="416"/>
+    <row customHeight="1" ht="16.5" r="417"/>
+    <row customHeight="1" ht="16.5" r="418"/>
+    <row customHeight="1" ht="16.5" r="419"/>
+    <row customHeight="1" ht="16.5" r="420"/>
+    <row customHeight="1" ht="16.5" r="421"/>
+    <row customHeight="1" ht="16.5" r="422"/>
+    <row customHeight="1" ht="16.5" r="423"/>
+    <row customHeight="1" ht="16.5" r="424"/>
+    <row customHeight="1" ht="16.5" r="425"/>
+    <row customHeight="1" ht="16.5" r="426"/>
+    <row customHeight="1" ht="16.5" r="427"/>
+    <row customHeight="1" ht="16.5" r="428"/>
+    <row customHeight="1" ht="16.5" r="429"/>
+    <row customHeight="1" ht="16.5" r="430"/>
+    <row customHeight="1" ht="16.5" r="431"/>
+    <row customHeight="1" ht="16.5" r="432"/>
+    <row customHeight="1" ht="16.5" r="433"/>
+    <row customHeight="1" ht="16.5" r="434"/>
+    <row customHeight="1" ht="16.5" r="435"/>
+    <row customHeight="1" ht="16.5" r="436"/>
+    <row customHeight="1" ht="16.5" r="437"/>
+    <row customHeight="1" ht="16.5" r="438"/>
+    <row customHeight="1" ht="16.5" r="439"/>
+    <row customHeight="1" ht="16.5" r="440"/>
+    <row customHeight="1" ht="16.5" r="441"/>
+    <row customHeight="1" ht="16.5" r="442"/>
+    <row customHeight="1" ht="16.5" r="443"/>
+    <row customHeight="1" ht="16.5" r="444"/>
+    <row customHeight="1" ht="16.5" r="445"/>
+    <row customHeight="1" ht="16.5" r="446"/>
+    <row customHeight="1" ht="16.5" r="447"/>
+    <row customHeight="1" ht="16.5" r="448"/>
+    <row customHeight="1" ht="16.5" r="449"/>
+    <row customHeight="1" ht="16.5" r="450"/>
+    <row customHeight="1" ht="16.5" r="451"/>
+    <row customHeight="1" ht="16.5" r="452"/>
+    <row customHeight="1" ht="16.5" r="453"/>
+    <row customHeight="1" ht="16.5" r="454"/>
+    <row customHeight="1" ht="16.5" r="455"/>
+    <row customHeight="1" ht="16.5" r="456"/>
+    <row customHeight="1" ht="16.5" r="457"/>
+    <row customHeight="1" ht="16.5" r="458"/>
+    <row customHeight="1" ht="16.5" r="459"/>
+    <row customHeight="1" ht="16.5" r="460"/>
+    <row customHeight="1" ht="16.5" r="461"/>
+    <row customHeight="1" ht="16.5" r="462"/>
+    <row customHeight="1" ht="16.5" r="463"/>
+    <row customHeight="1" ht="16.5" r="464"/>
+    <row customHeight="1" ht="16.5" r="465"/>
+    <row customHeight="1" ht="16.5" r="466"/>
+    <row customHeight="1" ht="16.5" r="467"/>
+    <row customHeight="1" ht="16.5" r="468"/>
+    <row customHeight="1" ht="16.5" r="469"/>
+    <row customHeight="1" ht="16.5" r="470"/>
+    <row customHeight="1" ht="16.5" r="471"/>
+    <row customHeight="1" ht="16.5" r="472"/>
+    <row customHeight="1" ht="16.5" r="473"/>
+    <row customHeight="1" ht="16.5" r="474"/>
+    <row customHeight="1" ht="16.5" r="475"/>
+    <row customHeight="1" ht="16.5" r="476"/>
+    <row customHeight="1" ht="16.5" r="477"/>
+    <row customHeight="1" ht="16.5" r="478"/>
+    <row customHeight="1" ht="16.5" r="479"/>
+    <row customHeight="1" ht="16.5" r="480"/>
+    <row customHeight="1" ht="16.5" r="481"/>
+    <row customHeight="1" ht="16.5" r="482"/>
+    <row customHeight="1" ht="16.5" r="483"/>
+    <row customHeight="1" ht="16.5" r="484"/>
+    <row customHeight="1" ht="16.5" r="485"/>
+    <row customHeight="1" ht="16.5" r="486"/>
+    <row customHeight="1" ht="16.5" r="487"/>
+    <row customHeight="1" ht="16.5" r="488"/>
+    <row customHeight="1" ht="16.5" r="489"/>
   </sheetData>
   <autoFilter ref="A1:AP488"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -1330,7 +1759,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA2" s="44" t="n">
+      <c r="AA2" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB2" t="n">
@@ -1347,7 +1776,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="AI2" s="44" t="n">
+      <c r="AI2" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ2" t="n">
@@ -1480,7 +1909,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA3" s="44" t="n">
+      <c r="AA3" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB3" t="n">
@@ -1497,7 +1926,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="AI3" s="44" t="n">
+      <c r="AI3" s="46" t="n">
         <v>44514</v>
       </c>
       <c r="AJ3" t="n">
@@ -1529,7 +1958,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>I962690000002BE</t>
         </is>
@@ -1630,7 +2059,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA4" s="44" t="n">
+      <c r="AA4" s="46" t="n">
         <v>44509</v>
       </c>
       <c r="AB4" t="n">
@@ -1647,7 +2076,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="AI4" s="44" t="n">
+      <c r="AI4" s="46" t="n">
         <v>44503</v>
       </c>
       <c r="AJ4" t="n">
@@ -1679,7 +2108,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>I962690000002BE</t>
         </is>
@@ -1780,7 +2209,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA5" s="44" t="n">
+      <c r="AA5" s="46" t="n">
         <v>44509</v>
       </c>
       <c r="AB5" t="n">
@@ -1797,7 +2226,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="AI5" s="44" t="n">
+      <c r="AI5" s="46" t="n">
         <v>44503</v>
       </c>
       <c r="AJ5" t="n">
@@ -1829,7 +2258,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>I962690000002BE</t>
         </is>
@@ -1930,7 +2359,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA6" s="44" t="n">
+      <c r="AA6" s="46" t="n">
         <v>44509</v>
       </c>
       <c r="AB6" t="n">
@@ -1947,7 +2376,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="AI6" s="44" t="n">
+      <c r="AI6" s="46" t="n">
         <v>44503</v>
       </c>
       <c r="AJ6" t="n">
@@ -1979,7 +2408,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>I962690000002BE</t>
         </is>
@@ -2080,7 +2509,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA7" s="44" t="n">
+      <c r="AA7" s="46" t="n">
         <v>44509</v>
       </c>
       <c r="AB7" t="n">
@@ -2097,7 +2526,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="AI7" s="44" t="n">
+      <c r="AI7" s="46" t="n">
         <v>44503</v>
       </c>
       <c r="AJ7" t="n">
@@ -2129,7 +2558,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>I962690000002BE</t>
         </is>
@@ -2230,7 +2659,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA8" s="44" t="n">
+      <c r="AA8" s="46" t="n">
         <v>44509</v>
       </c>
       <c r="AB8" t="n">
@@ -2247,7 +2676,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="AI8" s="44" t="n">
+      <c r="AI8" s="46" t="n">
         <v>44503</v>
       </c>
       <c r="AJ8" t="n">
@@ -2380,7 +2809,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA9" s="44" t="n">
+      <c r="AA9" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB9" t="n">
@@ -2402,7 +2831,7 @@
           <t>EJDPC@YAHOO.COM</t>
         </is>
       </c>
-      <c r="AI9" s="44" t="n">
+      <c r="AI9" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ9" t="n">
@@ -2434,7 +2863,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>I990036000001RT</t>
         </is>
@@ -2535,7 +2964,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA10" s="44" t="n">
+      <c r="AA10" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB10" t="n">
@@ -2557,7 +2986,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI10" s="44" t="n">
+      <c r="AI10" s="46" t="n">
         <v>44531</v>
       </c>
       <c r="AJ10" t="n">
@@ -2685,7 +3114,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA11" s="44" t="n">
+      <c r="AA11" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB11" t="n">
@@ -2707,7 +3136,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI11" s="44" t="n">
+      <c r="AI11" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ11" t="n">
@@ -2835,7 +3264,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA12" s="44" t="n">
+      <c r="AA12" s="46" t="n">
         <v>44512</v>
       </c>
       <c r="AB12" t="n">
@@ -2857,7 +3286,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI12" s="44" t="n">
+      <c r="AI12" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ12" t="n">
@@ -2884,7 +3313,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>I990223000001RT</t>
         </is>
@@ -2985,7 +3414,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA13" s="44" t="n">
+      <c r="AA13" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB13" t="n">
@@ -3007,7 +3436,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI13" s="44" t="n">
+      <c r="AI13" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ13" t="n">
@@ -3034,7 +3463,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>I990223000001RT</t>
         </is>
@@ -3135,7 +3564,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA14" s="44" t="n">
+      <c r="AA14" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB14" t="n">
@@ -3157,7 +3586,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI14" s="44" t="n">
+      <c r="AI14" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ14" t="n">
@@ -3285,7 +3714,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA15" s="44" t="n">
+      <c r="AA15" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB15" t="n">
@@ -3307,7 +3736,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI15" s="44" t="n">
+      <c r="AI15" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ15" t="n">
@@ -3334,7 +3763,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>I990036000001RT</t>
         </is>
@@ -3435,7 +3864,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA16" s="44" t="n">
+      <c r="AA16" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB16" t="n">
@@ -3457,7 +3886,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI16" s="44" t="n">
+      <c r="AI16" s="46" t="n">
         <v>44531</v>
       </c>
       <c r="AJ16" t="n">
@@ -3585,7 +4014,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA17" s="44" t="n">
+      <c r="AA17" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB17" t="n">
@@ -3607,7 +4036,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI17" s="44" t="n">
+      <c r="AI17" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ17" t="n">
@@ -3735,7 +4164,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA18" s="44" t="n">
+      <c r="AA18" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB18" t="n">
@@ -3757,7 +4186,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI18" s="44" t="n">
+      <c r="AI18" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ18" t="n">
@@ -3885,7 +4314,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA19" s="44" t="n">
+      <c r="AA19" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB19" t="n">
@@ -3907,7 +4336,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI19" s="44" t="n">
+      <c r="AI19" s="46" t="n">
         <v>44531</v>
       </c>
       <c r="AJ19" t="n">
@@ -4035,7 +4464,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA20" s="44" t="n">
+      <c r="AA20" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB20" t="n">
@@ -4057,7 +4486,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI20" s="44" t="n">
+      <c r="AI20" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ20" t="n">
@@ -4185,7 +4614,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA21" s="44" t="n">
+      <c r="AA21" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB21" t="n">
@@ -4207,7 +4636,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI21" s="44" t="n">
+      <c r="AI21" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ21" t="n">
@@ -4335,7 +4764,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA22" s="44" t="n">
+      <c r="AA22" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB22" t="n">
@@ -4357,7 +4786,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI22" s="44" t="n">
+      <c r="AI22" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ22" t="n">
@@ -4485,7 +4914,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA23" s="44" t="n">
+      <c r="AA23" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB23" t="n">
@@ -4507,7 +4936,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI23" s="44" t="n">
+      <c r="AI23" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ23" t="n">
@@ -4635,7 +5064,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA24" s="44" t="n">
+      <c r="AA24" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB24" t="n">
@@ -4657,7 +5086,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI24" s="44" t="n">
+      <c r="AI24" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ24" t="n">
@@ -4785,7 +5214,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA25" s="44" t="n">
+      <c r="AA25" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB25" t="n">
@@ -4812,7 +5241,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI25" s="44" t="n">
+      <c r="AI25" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ25" t="n">
@@ -4940,7 +5369,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA26" s="44" t="n">
+      <c r="AA26" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB26" t="n">
@@ -4962,7 +5391,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI26" s="44" t="n">
+      <c r="AI26" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ26" t="n">
@@ -5090,7 +5519,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA27" s="44" t="n">
+      <c r="AA27" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB27" t="n">
@@ -5112,7 +5541,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI27" s="44" t="n">
+      <c r="AI27" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ27" t="n">
@@ -5240,7 +5669,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA28" s="44" t="n">
+      <c r="AA28" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB28" t="n">
@@ -5262,7 +5691,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI28" s="44" t="n">
+      <c r="AI28" s="46" t="n">
         <v>44531</v>
       </c>
       <c r="AJ28" t="n">
@@ -5313,7 +5742,7 @@
       <c r="F29" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="45" t="n">
+      <c r="G29" s="48" t="n">
         <v>20</v>
       </c>
       <c r="H29" t="n">
@@ -5390,7 +5819,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA29" s="44" t="n">
+      <c r="AA29" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB29" t="n">
@@ -5412,7 +5841,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI29" s="44" t="n">
+      <c r="AI29" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ29" t="n">
@@ -5439,7 +5868,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="47" t="inlineStr">
         <is>
           <t>I991174000002RT</t>
         </is>
@@ -5463,7 +5892,7 @@
       <c r="F30" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="45" t="n">
+      <c r="G30" s="48" t="n">
         <v>20</v>
       </c>
       <c r="H30" t="n">
@@ -5540,7 +5969,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA30" s="44" t="n">
+      <c r="AA30" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB30" t="n">
@@ -5562,7 +5991,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI30" s="44" t="n">
+      <c r="AI30" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ30" t="n">
@@ -5613,7 +6042,7 @@
       <c r="F31" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="45" t="n">
+      <c r="G31" s="48" t="n">
         <v>20</v>
       </c>
       <c r="H31" t="n">
@@ -5690,7 +6119,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA31" s="44" t="n">
+      <c r="AA31" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB31" t="n">
@@ -5712,7 +6141,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI31" s="44" t="n">
+      <c r="AI31" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ31" t="n">
@@ -5739,7 +6168,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="47" t="inlineStr">
         <is>
           <t>I990222000002RT</t>
         </is>
@@ -5763,7 +6192,7 @@
       <c r="F32" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="45" t="n">
+      <c r="G32" s="48" t="n">
         <v>20</v>
       </c>
       <c r="H32" t="n">
@@ -5840,7 +6269,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA32" s="44" t="n">
+      <c r="AA32" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB32" t="n">
@@ -5862,7 +6291,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI32" s="44" t="n">
+      <c r="AI32" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ32" t="n">
@@ -5990,7 +6419,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA33" s="44" t="n">
+      <c r="AA33" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB33" t="n">
@@ -6012,7 +6441,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI33" s="44" t="n">
+      <c r="AI33" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ33" t="n">
@@ -6039,7 +6468,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="47" t="inlineStr">
         <is>
           <t>I991174000002RT</t>
         </is>
@@ -6063,7 +6492,7 @@
       <c r="F34" t="n">
         <v>2</v>
       </c>
-      <c r="G34" s="45" t="n">
+      <c r="G34" s="48" t="n">
         <v>10</v>
       </c>
       <c r="H34" t="n">
@@ -6140,7 +6569,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA34" s="44" t="n">
+      <c r="AA34" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB34" t="n">
@@ -6162,7 +6591,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI34" s="44" t="n">
+      <c r="AI34" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ34" t="n">
@@ -6213,7 +6642,7 @@
       <c r="F35" t="n">
         <v>2</v>
       </c>
-      <c r="G35" s="45" t="n">
+      <c r="G35" s="48" t="n">
         <v>10</v>
       </c>
       <c r="H35" t="n">
@@ -6290,7 +6719,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA35" s="44" t="n">
+      <c r="AA35" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB35" t="n">
@@ -6312,7 +6741,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI35" s="44" t="n">
+      <c r="AI35" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ35" t="n">
@@ -6339,7 +6768,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="47" t="inlineStr">
         <is>
           <t>I990222000002RT</t>
         </is>
@@ -6363,7 +6792,7 @@
       <c r="F36" t="n">
         <v>2</v>
       </c>
-      <c r="G36" s="45" t="n">
+      <c r="G36" s="48" t="n">
         <v>10</v>
       </c>
       <c r="H36" t="n">
@@ -6440,7 +6869,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA36" s="44" t="n">
+      <c r="AA36" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB36" t="n">
@@ -6462,7 +6891,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI36" s="44" t="n">
+      <c r="AI36" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ36" t="n">
@@ -6590,7 +7019,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA37" s="44" t="n">
+      <c r="AA37" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB37" t="n">
@@ -6612,7 +7041,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI37" s="44" t="n">
+      <c r="AI37" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ37" t="n">
@@ -6663,7 +7092,7 @@
       <c r="F38" t="n">
         <v>2</v>
       </c>
-      <c r="G38" s="45" t="n">
+      <c r="G38" s="48" t="n">
         <v>8</v>
       </c>
       <c r="H38" t="n">
@@ -6745,7 +7174,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA38" s="44" t="n">
+      <c r="AA38" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB38" t="n">
@@ -6767,7 +7196,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI38" s="44" t="n">
+      <c r="AI38" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ38" t="n">
@@ -6895,7 +7324,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA39" s="44" t="n">
+      <c r="AA39" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB39" t="n">
@@ -6917,7 +7346,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI39" s="44" t="n">
+      <c r="AI39" s="46" t="n">
         <v>44524</v>
       </c>
       <c r="AJ39" t="n">
@@ -7045,7 +7474,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA40" s="44" t="n">
+      <c r="AA40" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB40" t="n">
@@ -7067,7 +7496,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI40" s="44" t="n">
+      <c r="AI40" s="46" t="n">
         <v>44524</v>
       </c>
       <c r="AJ40" t="n">
@@ -7191,7 +7620,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA41" s="44" t="n">
+      <c r="AA41" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB41" t="n">
@@ -7213,7 +7642,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI41" s="44" t="n">
+      <c r="AI41" s="46" t="n">
         <v>44524</v>
       </c>
       <c r="AJ41" t="n">
@@ -7341,7 +7770,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA42" s="44" t="n">
+      <c r="AA42" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB42" t="n">
@@ -7363,7 +7792,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI42" s="44" t="n">
+      <c r="AI42" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ42" t="n">
@@ -7414,7 +7843,7 @@
       <c r="F43" t="n">
         <v>2</v>
       </c>
-      <c r="G43" s="45" t="n">
+      <c r="G43" s="48" t="n">
         <v>3</v>
       </c>
       <c r="H43" t="n">
@@ -7487,7 +7916,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA43" s="44" t="n">
+      <c r="AA43" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB43" t="n">
@@ -7509,7 +7938,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI43" s="44" t="n">
+      <c r="AI43" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ43" t="n">
@@ -7637,7 +8066,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA44" s="44" t="n">
+      <c r="AA44" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB44" t="n">
@@ -7659,7 +8088,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI44" s="44" t="n">
+      <c r="AI44" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ44" t="n">
@@ -7783,7 +8212,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA45" s="44" t="n">
+      <c r="AA45" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB45" t="n">
@@ -7805,7 +8234,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI45" s="44" t="n">
+      <c r="AI45" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ45" t="n">
@@ -7856,7 +8285,7 @@
       <c r="F46" t="n">
         <v>3</v>
       </c>
-      <c r="G46" s="45" t="n">
+      <c r="G46" s="48" t="n">
         <v>9</v>
       </c>
       <c r="H46" t="n">
@@ -7933,7 +8362,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA46" s="44" t="n">
+      <c r="AA46" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB46" t="n">
@@ -7955,7 +8384,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI46" s="44" t="n">
+      <c r="AI46" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ46" t="n">
@@ -8083,7 +8512,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA47" s="44" t="n">
+      <c r="AA47" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB47" t="n">
@@ -8105,7 +8534,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI47" s="44" t="n">
+      <c r="AI47" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ47" t="n">
@@ -8233,7 +8662,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA48" s="44" t="n">
+      <c r="AA48" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB48" t="n">
@@ -8255,7 +8684,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI48" s="44" t="n">
+      <c r="AI48" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ48" t="n">
@@ -8306,7 +8735,7 @@
       <c r="F49" t="n">
         <v>2</v>
       </c>
-      <c r="G49" s="45" t="n">
+      <c r="G49" s="48" t="n">
         <v>3</v>
       </c>
       <c r="H49" t="n">
@@ -8379,7 +8808,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA49" s="44" t="n">
+      <c r="AA49" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB49" t="n">
@@ -8401,7 +8830,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI49" s="44" t="n">
+      <c r="AI49" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ49" t="n">
@@ -8529,7 +8958,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA50" s="44" t="n">
+      <c r="AA50" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB50" t="n">
@@ -8551,7 +8980,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI50" s="44" t="n">
+      <c r="AI50" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ50" t="n">
@@ -8679,7 +9108,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA51" s="44" t="n">
+      <c r="AA51" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB51" t="n">
@@ -8701,7 +9130,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI51" s="44" t="n">
+      <c r="AI51" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ51" t="n">
@@ -8825,7 +9254,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA52" s="44" t="n">
+      <c r="AA52" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB52" t="n">
@@ -8847,7 +9276,7 @@
           <t>SHIP VIA FEDERAL EX-GROUND</t>
         </is>
       </c>
-      <c r="AI52" s="44" t="n">
+      <c r="AI52" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ52" t="n">
@@ -8874,7 +9303,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="47" t="inlineStr">
         <is>
           <t>I991186000001FE</t>
         </is>
@@ -8971,7 +9400,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA53" s="44" t="n">
+      <c r="AA53" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB53" t="n">
@@ -8993,7 +9422,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI53" s="44" t="n">
+      <c r="AI53" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ53" t="n">
@@ -9020,7 +9449,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="47" t="inlineStr">
         <is>
           <t>I991182000001FE</t>
         </is>
@@ -9044,7 +9473,7 @@
       <c r="F54" t="n">
         <v>3</v>
       </c>
-      <c r="G54" s="45" t="n">
+      <c r="G54" s="48" t="n">
         <v>9</v>
       </c>
       <c r="H54" t="n">
@@ -9121,7 +9550,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA54" s="44" t="n">
+      <c r="AA54" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB54" t="n">
@@ -9143,7 +9572,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI54" s="44" t="n">
+      <c r="AI54" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ54" t="n">
@@ -9271,7 +9700,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA55" s="44" t="n">
+      <c r="AA55" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB55" t="n">
@@ -9293,7 +9722,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI55" s="44" t="n">
+      <c r="AI55" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ55" t="n">
@@ -9417,7 +9846,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA56" s="44" t="n">
+      <c r="AA56" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB56" t="n">
@@ -9439,7 +9868,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI56" s="44" t="n">
+      <c r="AI56" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ56" t="n">
@@ -9563,7 +9992,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA57" s="44" t="n">
+      <c r="AA57" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB57" t="n">
@@ -9585,7 +10014,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI57" s="44" t="n">
+      <c r="AI57" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ57" t="n">
@@ -9713,7 +10142,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA58" s="44" t="n">
+      <c r="AA58" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB58" t="n">
@@ -9735,7 +10164,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI58" s="44" t="n">
+      <c r="AI58" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ58" t="n">
@@ -9863,7 +10292,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA59" s="44" t="n">
+      <c r="AA59" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB59" t="n">
@@ -9885,7 +10314,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI59" s="44" t="n">
+      <c r="AI59" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ59" t="n">
@@ -9936,7 +10365,7 @@
       <c r="F60" t="n">
         <v>3</v>
       </c>
-      <c r="G60" s="45" t="n">
+      <c r="G60" s="48" t="n">
         <v>3</v>
       </c>
       <c r="H60" t="n">
@@ -10009,7 +10438,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA60" s="44" t="n">
+      <c r="AA60" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB60" t="n">
@@ -10031,7 +10460,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI60" s="44" t="n">
+      <c r="AI60" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ60" t="n">
@@ -10082,7 +10511,7 @@
       <c r="F61" t="n">
         <v>2</v>
       </c>
-      <c r="G61" s="45" t="n">
+      <c r="G61" s="48" t="n">
         <v>3</v>
       </c>
       <c r="H61" t="n">
@@ -10159,7 +10588,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA61" s="44" t="n">
+      <c r="AA61" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB61" t="n">
@@ -10181,7 +10610,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI61" s="44" t="n">
+      <c r="AI61" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ61" t="n">
@@ -10232,7 +10661,7 @@
       <c r="F62" t="n">
         <v>2</v>
       </c>
-      <c r="G62" s="45" t="n">
+      <c r="G62" s="48" t="n">
         <v>3</v>
       </c>
       <c r="H62" t="n">
@@ -10314,7 +10743,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA62" s="44" t="n">
+      <c r="AA62" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB62" t="n">
@@ -10336,7 +10765,7 @@
           <t>SHIP VIA FEDEX GND</t>
         </is>
       </c>
-      <c r="AI62" s="44" t="n">
+      <c r="AI62" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ62" t="n">
@@ -10387,7 +10816,7 @@
       <c r="F63" t="n">
         <v>2</v>
       </c>
-      <c r="G63" s="45" t="n">
+      <c r="G63" s="48" t="n">
         <v>3</v>
       </c>
       <c r="H63" t="n">
@@ -10469,7 +10898,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA63" s="44" t="n">
+      <c r="AA63" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB63" t="n">
@@ -10491,7 +10920,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI63" s="44" t="n">
+      <c r="AI63" s="46" t="n">
         <v>44531</v>
       </c>
       <c r="AJ63" t="n">
@@ -10619,7 +11048,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA64" s="44" t="n">
+      <c r="AA64" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB64" t="n">
@@ -10641,7 +11070,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI64" s="44" t="n">
+      <c r="AI64" s="46" t="n">
         <v>44531</v>
       </c>
       <c r="AJ64" t="n">
@@ -10769,7 +11198,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA65" s="44" t="n">
+      <c r="AA65" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB65" t="n">
@@ -10791,7 +11220,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI65" s="44" t="n">
+      <c r="AI65" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ65" t="n">
@@ -10842,7 +11271,7 @@
       <c r="F66" t="n">
         <v>2</v>
       </c>
-      <c r="G66" s="45" t="n">
+      <c r="G66" s="48" t="n">
         <v>1</v>
       </c>
       <c r="H66" t="n">
@@ -10924,7 +11353,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA66" s="44" t="n">
+      <c r="AA66" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB66" t="n">
@@ -10946,7 +11375,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI66" s="44" t="n">
+      <c r="AI66" s="46" t="n">
         <v>44532</v>
       </c>
       <c r="AJ66" t="n">
@@ -11074,7 +11503,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA67" s="44" t="n">
+      <c r="AA67" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB67" t="n">
@@ -11101,7 +11530,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI67" s="44" t="n">
+      <c r="AI67" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ67" t="n">
@@ -11229,7 +11658,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA68" s="44" t="n">
+      <c r="AA68" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB68" t="n">
@@ -11251,7 +11680,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI68" s="44" t="n">
+      <c r="AI68" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ68" t="n">
@@ -11379,7 +11808,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA69" s="44" t="n">
+      <c r="AA69" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB69" t="n">
@@ -11401,7 +11830,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI69" s="44" t="n">
+      <c r="AI69" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ69" t="n">
@@ -11529,7 +11958,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA70" s="44" t="n">
+      <c r="AA70" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB70" t="n">
@@ -11551,7 +11980,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI70" s="44" t="n">
+      <c r="AI70" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ70" t="n">
@@ -11679,7 +12108,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA71" s="44" t="n">
+      <c r="AA71" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB71" t="n">
@@ -11701,7 +12130,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY FEDH</t>
         </is>
       </c>
-      <c r="AI71" s="44" t="n">
+      <c r="AI71" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ71" t="n">
@@ -11728,7 +12157,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="47" t="inlineStr">
         <is>
           <t>I990036000001RT</t>
         </is>
@@ -11829,7 +12258,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA72" s="44" t="n">
+      <c r="AA72" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB72" t="n">
@@ -11851,7 +12280,7 @@
           <t>SHIP VIA FEDEX HOME DELV</t>
         </is>
       </c>
-      <c r="AI72" s="44" t="n">
+      <c r="AI72" s="46" t="n">
         <v>44531</v>
       </c>
       <c r="AJ72" t="n">
@@ -11878,7 +12307,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="47" t="inlineStr">
         <is>
           <t>I991182000001FE</t>
         </is>
@@ -11902,7 +12331,7 @@
       <c r="F73" t="n">
         <v>3</v>
       </c>
-      <c r="G73" s="45" t="n">
+      <c r="G73" s="48" t="n">
         <v>9</v>
       </c>
       <c r="H73" t="n">
@@ -11979,7 +12408,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA73" s="44" t="n">
+      <c r="AA73" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB73" t="n">
@@ -12001,7 +12430,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI73" s="44" t="n">
+      <c r="AI73" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ73" t="n">
@@ -12028,7 +12457,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="47" t="inlineStr">
         <is>
           <t>I991182000001FE</t>
         </is>
@@ -12052,7 +12481,7 @@
       <c r="F74" t="n">
         <v>2</v>
       </c>
-      <c r="G74" s="45" t="n">
+      <c r="G74" s="48" t="n">
         <v>6</v>
       </c>
       <c r="H74" t="n">
@@ -12129,7 +12558,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA74" s="44" t="n">
+      <c r="AA74" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB74" t="n">
@@ -12151,7 +12580,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI74" s="44" t="n">
+      <c r="AI74" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ74" t="n">
@@ -12202,7 +12631,7 @@
       <c r="F75" t="n">
         <v>3</v>
       </c>
-      <c r="G75" s="45" t="n">
+      <c r="G75" s="48" t="n">
         <v>9</v>
       </c>
       <c r="H75" t="n">
@@ -12279,7 +12708,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA75" s="44" t="n">
+      <c r="AA75" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB75" t="n">
@@ -12301,7 +12730,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI75" s="44" t="n">
+      <c r="AI75" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ75" t="n">
@@ -12352,7 +12781,7 @@
       <c r="F76" t="n">
         <v>3</v>
       </c>
-      <c r="G76" s="45" t="n">
+      <c r="G76" s="48" t="n">
         <v>9</v>
       </c>
       <c r="H76" t="n">
@@ -12429,7 +12858,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA76" s="44" t="n">
+      <c r="AA76" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB76" t="n">
@@ -12451,7 +12880,7 @@
           <t>SHIP VIA FEDERAL EX-STANDARD GROUND</t>
         </is>
       </c>
-      <c r="AI76" s="44" t="n">
+      <c r="AI76" s="46" t="n">
         <v>44523</v>
       </c>
       <c r="AJ76" t="n">
@@ -12805,7 +13234,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA2" s="44" t="n">
+      <c r="AA2" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB2" t="n">
@@ -12827,7 +13256,7 @@
           <t>SHIP VIA Ground</t>
         </is>
       </c>
-      <c r="AI2" s="44" t="n">
+      <c r="AI2" s="46" t="n">
         <v>44515</v>
       </c>
       <c r="AJ2" t="n">
@@ -12955,7 +13384,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA3" s="44" t="n">
+      <c r="AA3" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB3" t="n">
@@ -12977,7 +13406,7 @@
           <t>SHIP VIA Ground</t>
         </is>
       </c>
-      <c r="AI3" s="44" t="n">
+      <c r="AI3" s="46" t="n">
         <v>44513</v>
       </c>
       <c r="AJ3" t="n">
@@ -13110,7 +13539,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA4" s="44" t="n">
+      <c r="AA4" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB4" t="n">
@@ -13132,7 +13561,7 @@
           <t>SHIP VIA Ground</t>
         </is>
       </c>
-      <c r="AI4" s="44" t="n">
+      <c r="AI4" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ4" t="n">
@@ -13260,7 +13689,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA5" s="44" t="n">
+      <c r="AA5" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB5" t="n">
@@ -13282,7 +13711,7 @@
           <t>SHIP VIA Ground</t>
         </is>
       </c>
-      <c r="AI5" s="44" t="n">
+      <c r="AI5" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ5" t="n">
@@ -13410,7 +13839,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA6" s="44" t="n">
+      <c r="AA6" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB6" t="n">
@@ -13432,7 +13861,7 @@
           <t>SHIP VIA Ground</t>
         </is>
       </c>
-      <c r="AI6" s="44" t="n">
+      <c r="AI6" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ6" t="n">
@@ -13685,7 +14114,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="47" t="inlineStr">
         <is>
           <t>I991143000001RT</t>
         </is>
@@ -13782,7 +14211,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA2" s="44" t="n">
+      <c r="AA2" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB2" t="n">
@@ -13804,7 +14233,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI2" s="44" t="n">
+      <c r="AI2" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ2" t="n">
@@ -13831,7 +14260,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>I989848000001RT</t>
         </is>
@@ -13928,7 +14357,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA3" s="44" t="n">
+      <c r="AA3" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB3" t="n">
@@ -13950,7 +14379,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI3" s="44" t="n">
+      <c r="AI3" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ3" t="n">
@@ -14074,7 +14503,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA4" s="44" t="n">
+      <c r="AA4" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB4" t="n">
@@ -14096,7 +14525,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI4" s="44" t="n">
+      <c r="AI4" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ4" t="n">
@@ -14123,7 +14552,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>I991143000001RT</t>
         </is>
@@ -14220,7 +14649,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA5" s="44" t="n">
+      <c r="AA5" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB5" t="n">
@@ -14242,7 +14671,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI5" s="44" t="n">
+      <c r="AI5" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ5" t="n">
@@ -14269,7 +14698,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>I989848000001RT</t>
         </is>
@@ -14366,7 +14795,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA6" s="44" t="n">
+      <c r="AA6" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB6" t="n">
@@ -14388,7 +14817,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI6" s="44" t="n">
+      <c r="AI6" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ6" t="n">
@@ -14512,7 +14941,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA7" s="44" t="n">
+      <c r="AA7" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB7" t="n">
@@ -14534,7 +14963,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI7" s="44" t="n">
+      <c r="AI7" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ7" t="n">
@@ -14658,7 +15087,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA8" s="44" t="n">
+      <c r="AA8" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB8" t="n">
@@ -14680,7 +15109,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI8" s="44" t="n">
+      <c r="AI8" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ8" t="n">
@@ -14804,7 +15233,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA9" s="44" t="n">
+      <c r="AA9" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB9" t="n">
@@ -14826,7 +15255,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI9" s="44" t="n">
+      <c r="AI9" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ9" t="n">
@@ -14950,7 +15379,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA10" s="44" t="n">
+      <c r="AA10" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB10" t="n">
@@ -14972,7 +15401,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI10" s="44" t="n">
+      <c r="AI10" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ10" t="n">
@@ -15096,7 +15525,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA11" s="44" t="n">
+      <c r="AA11" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB11" t="n">
@@ -15118,7 +15547,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI11" s="44" t="n">
+      <c r="AI11" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ11" t="n">
@@ -15242,7 +15671,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA12" s="44" t="n">
+      <c r="AA12" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB12" t="n">
@@ -15264,7 +15693,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI12" s="44" t="n">
+      <c r="AI12" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ12" t="n">
@@ -15388,7 +15817,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA13" s="44" t="n">
+      <c r="AA13" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB13" t="n">
@@ -15410,7 +15839,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI13" s="44" t="n">
+      <c r="AI13" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ13" t="n">
@@ -15534,7 +15963,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA14" s="44" t="n">
+      <c r="AA14" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB14" t="n">
@@ -15556,7 +15985,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI14" s="44" t="n">
+      <c r="AI14" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ14" t="n">
@@ -15685,7 +16114,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA15" s="44" t="n">
+      <c r="AA15" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB15" t="n">
@@ -15707,7 +16136,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI15" s="44" t="n">
+      <c r="AI15" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ15" t="n">
@@ -15831,7 +16260,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA16" s="44" t="n">
+      <c r="AA16" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB16" t="n">
@@ -15853,7 +16282,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI16" s="44" t="n">
+      <c r="AI16" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ16" t="n">
@@ -15880,7 +16309,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="47" t="inlineStr">
         <is>
           <t>I989848000001RT</t>
         </is>
@@ -15977,7 +16406,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA17" s="44" t="n">
+      <c r="AA17" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB17" t="n">
@@ -15999,7 +16428,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI17" s="44" t="n">
+      <c r="AI17" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ17" t="n">
@@ -16026,7 +16455,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="47" t="inlineStr">
         <is>
           <t>I991143000001RT</t>
         </is>
@@ -16123,7 +16552,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA18" s="44" t="n">
+      <c r="AA18" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB18" t="n">
@@ -16145,7 +16574,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI18" s="44" t="n">
+      <c r="AI18" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ18" t="n">
@@ -16172,7 +16601,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>I991143000001RT</t>
         </is>
@@ -16269,7 +16698,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA19" s="44" t="n">
+      <c r="AA19" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB19" t="n">
@@ -16291,7 +16720,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI19" s="44" t="n">
+      <c r="AI19" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ19" t="n">
@@ -16415,7 +16844,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA20" s="44" t="n">
+      <c r="AA20" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB20" t="n">
@@ -16437,7 +16866,7 @@
           <t>SHIP VIA FEDEX HOME DELIVERY</t>
         </is>
       </c>
-      <c r="AI20" s="44" t="n">
+      <c r="AI20" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ20" t="n">
@@ -16690,7 +17119,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="47" t="inlineStr">
         <is>
           <t>I991610000001RT</t>
         </is>
@@ -16787,7 +17216,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA2" s="44" t="n">
+      <c r="AA2" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB2" t="n">
@@ -16809,7 +17238,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI2" s="44" t="n">
+      <c r="AI2" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ2" t="n">
@@ -16836,7 +17265,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>I990051000001RT</t>
         </is>
@@ -16933,7 +17362,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA3" s="44" t="n">
+      <c r="AA3" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB3" t="n">
@@ -16955,7 +17384,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI3" s="44" t="n">
+      <c r="AI3" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ3" t="n">
@@ -16982,7 +17411,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>I991610000001RT</t>
         </is>
@@ -17079,7 +17508,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA4" s="44" t="n">
+      <c r="AA4" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB4" t="n">
@@ -17101,7 +17530,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI4" s="44" t="n">
+      <c r="AI4" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ4" t="n">
@@ -17128,7 +17557,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>I990051000001RT</t>
         </is>
@@ -17225,7 +17654,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA5" s="44" t="n">
+      <c r="AA5" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB5" t="n">
@@ -17247,7 +17676,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI5" s="44" t="n">
+      <c r="AI5" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ5" t="n">
@@ -17274,7 +17703,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>I988288000001RT</t>
         </is>
@@ -17371,7 +17800,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA6" s="44" t="n">
+      <c r="AA6" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB6" t="n">
@@ -17398,7 +17827,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI6" s="44" t="n">
+      <c r="AI6" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AJ6" t="n">
@@ -17522,7 +17951,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA7" s="44" t="n">
+      <c r="AA7" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB7" t="n">
@@ -17544,7 +17973,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI7" s="44" t="n">
+      <c r="AI7" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ7" t="n">
@@ -17571,7 +18000,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>I990051000001RT</t>
         </is>
@@ -17668,7 +18097,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA8" s="44" t="n">
+      <c r="AA8" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB8" t="n">
@@ -17690,7 +18119,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI8" s="44" t="n">
+      <c r="AI8" s="46" t="n">
         <v>44518</v>
       </c>
       <c r="AJ8" t="n">
@@ -17814,7 +18243,7 @@
           <t>PROFILE</t>
         </is>
       </c>
-      <c r="AA9" s="44" t="n">
+      <c r="AA9" s="46" t="n">
         <v>44517</v>
       </c>
       <c r="AB9" t="n">
@@ -17836,7 +18265,7 @@
           <t>SHIP VIA UPS GROUND</t>
         </is>
       </c>
-      <c r="AI9" s="44" t="n">
+      <c r="AI9" s="46" t="n">
         <v>44519</v>
       </c>
       <c r="AJ9" t="n">

</xml_diff>